<commit_message>
Fixed issue with get_or_create_index service.
</commit_message>
<xml_diff>
--- a/backend/fms_core/tests/valid_templates/Index_creation_v3_7_0.xlsx
+++ b/backend/fms_core/tests/valid_templates/Index_creation_v3_7_0.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="48">
   <si>
     <t xml:space="preserve">Index Creation Template</t>
   </si>
@@ -1921,7 +1921,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U711"/>
-  <sheetFormatPr defaultColWidth="12.65625" defaultRowHeight="14" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6484375" defaultRowHeight="14" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.83"/>
@@ -2043,11 +2043,19 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>12</v>
+      </c>
       <c r="E12" s="17"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5059,8 +5067,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H386"/>
-  <sheetFormatPr defaultColWidth="12.65625" defaultRowHeight="14" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H1000"/>
+  <sheetFormatPr defaultColWidth="12.6484375" defaultRowHeight="14" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="233.66"/>

</xml_diff>